<commit_message>
Proje_Kontrol_Listesi has been updated
</commit_message>
<xml_diff>
--- a/Docs/Proje_Kontrol_Listesi.xlsx
+++ b/Docs/Proje_Kontrol_Listesi.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alpte\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ONAL\Documents\GitHub\Bil481Proje\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{659A62BE-050A-4640-804F-2EF431A73C02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F6344AE-23D5-4723-B0AB-C1E7A20637D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detayl__Kontrol_Listesi" sheetId="1" r:id="rId1"/>
@@ -553,9 +553,6 @@
     <t>Performans kriterleri tanimlanmistir: Buton tiklama veya veritabani sorgusuna &lt;2 saniye yanit süresi. Istatistik paneli verilerini &lt;=2 saniyede yüklemesi gerekmektedir.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tasarim kisitlari belirtilmistir: Java/JavaFX tabanli masaüstü gelistirme, SQLite yerel veritabani, offline çalışır, Maven ile derleme. Uygulama bulut/sunucu gerektirmez. </t>
-  </si>
-  <si>
     <t>Uygulama masaüstü (Windows)  cihazlarda çalisabilmelidir. JavaFX  kullanilmaktadir.</t>
   </si>
   <si>
@@ -566,6 +563,9 @@
   </si>
   <si>
     <t xml:space="preserve">Bütçe plani olusturulmustur: Tüm araçlar ücretsiz/açik kaynaklidir (Java, JavaFX, SQLite, GitHub, VSCode). </t>
+  </si>
+  <si>
+    <t>Tasarim kisitlari belirtilmistir: Java/JavaFX tabanli masaüstü gelistirme, SQLite yerel veritabani, offline çalışır, Maven ile derleme. Uygulama bulut/sunucu gerektirmez. Geliştirme sürecinde Claude 4.6 Sonnet, Github Copilot, Gemini 3.1 Pro yapay zekalarından faydalanılmıştır.</t>
   </si>
 </sst>
 </file>
@@ -928,17 +928,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F1000"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43" customWidth="1"/>
-    <col min="2" max="2" width="57.6640625" customWidth="1"/>
+    <col min="2" max="2" width="57.6328125" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
     <col min="4" max="4" width="90" customWidth="1"/>
-    <col min="5" max="5" width="23.33203125" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" customWidth="1"/>
+    <col min="5" max="5" width="23.36328125" customWidth="1"/>
+    <col min="6" max="6" width="24.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -947,7 +947,7 @@
       <c r="D1" s="2"/>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -956,7 +956,7 @@
       <c r="D2" s="2"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -974,7 +974,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
@@ -992,7 +992,7 @@
       </c>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>28</v>
       </c>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>32</v>
       </c>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>36</v>
       </c>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>40</v>
       </c>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>43</v>
       </c>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>46</v>
       </c>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>50</v>
       </c>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>53</v>
       </c>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>57</v>
       </c>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>62</v>
       </c>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>65</v>
       </c>
@@ -1273,14 +1273,14 @@
         <v>67</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>10</v>
       </c>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>68</v>
       </c>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>73</v>
       </c>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>77</v>
       </c>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>82</v>
       </c>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>87</v>
       </c>
@@ -1363,14 +1363,14 @@
         <v>89</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>90</v>
       </c>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>91</v>
       </c>
@@ -1381,14 +1381,14 @@
         <v>93</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>10</v>
       </c>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>94</v>
       </c>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>99</v>
       </c>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>103</v>
       </c>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>108</v>
       </c>
@@ -1453,14 +1453,14 @@
         <v>110</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>111</v>
       </c>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>112</v>
       </c>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>117</v>
       </c>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>120</v>
       </c>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>123</v>
       </c>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>127</v>
       </c>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>130</v>
       </c>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>134</v>
       </c>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>138</v>
       </c>
@@ -1597,14 +1597,14 @@
         <v>140</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>10</v>
       </c>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>141</v>
       </c>

</xml_diff>